<commit_message>
Updated broken links Excel file to use more specific clinics pages.
</commit_message>
<xml_diff>
--- a/website/home/migrations/0115_create_redirects_for_broken_pdf_links.xlsx
+++ b/website/home/migrations/0115_create_redirects_for_broken_pdf_links.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30023"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{70AA2362-466E-4544-9F64-EC84C8B140F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F74BE9C8-A254-4ABD-B8FE-8B7164039CA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
   <si>
     <t>From</t>
   </si>
@@ -48,7 +48,7 @@
     <t>/clinics_academic.htm</t>
   </si>
   <si>
-    <t>/clinics/</t>
+    <t>/clinics-academic/</t>
   </si>
   <si>
     <t>permanent</t>
@@ -57,7 +57,13 @@
     <t>/clinics_academic_nonlaw_school.htm</t>
   </si>
   <si>
+    <t>/clinics-acadmic-non-law-school/</t>
+  </si>
+  <si>
     <t>/clinics_nonacademic.htm</t>
+  </si>
+  <si>
+    <t>/clinics-nonacademic/</t>
   </si>
   <si>
     <t>/rules/judicial_misconduct_or_disability/jcd_complaint_form.pdf</t>
@@ -130,18 +136,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -170,17 +168,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -531,7 +527,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -539,10 +535,10 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -550,10 +546,10 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>
@@ -561,10 +557,10 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
@@ -572,10 +568,10 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
@@ -583,10 +579,10 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
         <v>6</v>
@@ -594,10 +590,10 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C9" t="s">
         <v>6</v>
@@ -605,10 +601,10 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
         <v>6</v>
@@ -616,10 +612,10 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C11" t="s">
         <v>6</v>
@@ -627,10 +623,10 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
         <v>6</v>
@@ -638,10 +634,10 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
         <v>6</v>
@@ -649,10 +645,10 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
         <v>6</v>
@@ -660,46 +656,16 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C15" t="s">
         <v>6</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="http://www.ustaxcourt.gov/clinics_academic.htm" xr:uid="{BC65B5DF-6FC4-42AF-9265-DA446B9A3A9E}"/>
-    <hyperlink ref="B2" r:id="rId2" display="https://www.ustaxcourt.gov/clinics/" xr:uid="{DF9A7520-137E-4553-A289-BAD7EAC5BD3E}"/>
-    <hyperlink ref="A3" r:id="rId3" display="http://www.ustaxcourt.gov/clinics_academic_nonlaw_school.htm" xr:uid="{E0382124-F2BC-4DF0-90F1-F93001A4B695}"/>
-    <hyperlink ref="B3" r:id="rId4" display="https://www.ustaxcourt.gov/clinics/" xr:uid="{D33FC480-154C-4187-B09B-776D1D16F1E2}"/>
-    <hyperlink ref="A4" r:id="rId5" display="http://www.ustaxcourt.gov/clinics_nonacademic.htm" xr:uid="{6D0297B4-93FE-479C-8972-2616367B441A}"/>
-    <hyperlink ref="B4" r:id="rId6" display="https://www.ustaxcourt.gov/clinics/" xr:uid="{0AF2B245-5C9F-4A8C-A0A3-C394462B45D4}"/>
-    <hyperlink ref="A5" r:id="rId7" display="http://www.ustaxcourt.gov/rules/judicial_misconduct_or_disability/jcd_complaint_form.pdf" xr:uid="{DF925E45-D6F9-44FF-9A17-2DF7A57C9635}"/>
-    <hyperlink ref="B5" r:id="rId8" display="https://ustaxcourt.gov/files/documents/jcd_complaint_form.pdf" xr:uid="{35A0BCFD-5487-4C5B-A272-6FB92D848C34}"/>
-    <hyperlink ref="A6" r:id="rId9" display="http://www.ustaxcourt.gov/rules/judicial_misconduct_or_disability/jcd_rules.pdf" xr:uid="{9EAF9F43-59F7-4550-9F50-D79BAEE33960}"/>
-    <hyperlink ref="B6" r:id="rId10" display="https://ustaxcourt.gov/files/documents/jcd_rules.pdf" xr:uid="{FDA32E4B-7F27-4210-BEE2-A260EFA2025E}"/>
-    <hyperlink ref="A7" r:id="rId11" display="https://www.ustaxcourt.gov/admin_orders/Admin_Order_No_2020-02.pdf" xr:uid="{A7754652-3025-45DD-B75D-1EE1B27FB9DB}"/>
-    <hyperlink ref="B7" r:id="rId12" display="https://ustaxcourt.gov/files/documents/Administrative_Order_2020-02.pdf" xr:uid="{38927A10-60F7-4A7A-9C26-5BC1F4CC24FB}"/>
-    <hyperlink ref="A8" r:id="rId13" display="https://www.ustaxcourt.gov/admin_orders/Admin_Order_No_2020-03.pdf" xr:uid="{8DC4D721-EACC-4D90-93A7-ED154388B9AF}"/>
-    <hyperlink ref="B8" r:id="rId14" display="https://ustaxcourt.gov/files/documents/Administrative_Order_2020-03.pdf" xr:uid="{AE772723-D16A-43D8-845E-051821B57054}"/>
-    <hyperlink ref="A9" r:id="rId15" display="https://www.ustaxcourt.gov/forms/Admission_Attorney_Form_30.pdf" xr:uid="{ED53D74E-2705-46B7-B71B-4EBCDF8890A0}"/>
-    <hyperlink ref="B9" r:id="rId16" display="https://ustaxcourt.gov/files/documents/Application_for_Admission_to_Practice_Attorney_Form_30.pdf" xr:uid="{1814B23C-3A09-4F63-8C7A-87E0E7009908}"/>
-    <hyperlink ref="A10" r:id="rId17" display="https://www.ustaxcourt.gov/forms/Notice_of_Completion_LEA.pdf" xr:uid="{CAA10D8C-9324-43AC-A9AB-93C00DB14A19}"/>
-    <hyperlink ref="B10" r:id="rId18" display="https://ustaxcourt.gov/files/documents/Notice_of_Completion_LEA.pdf" xr:uid="{E1E4BD9D-4A33-4290-9B61-6B283232DED2}"/>
-    <hyperlink ref="A11" r:id="rId19" display="https://www.ustaxcourt.gov/resources/administrative_orders/Administrative_Order_2021-02.pdf" xr:uid="{6B53C85B-A36F-41E5-AE32-94555D4A85DE}"/>
-    <hyperlink ref="B11" r:id="rId20" display="https://ustaxcourt.gov/files/documents/Administrative_Order_2022-01_Repealed.pdf" xr:uid="{63FC6B16-2D4C-4295-9690-1E33C3E904E1}"/>
-    <hyperlink ref="A12" r:id="rId21" display="https://www.ustaxcourt.gov/rules/Title_II.pdf" xr:uid="{E994BF62-5726-4D53-9392-541B23B78019}"/>
-    <hyperlink ref="B12" r:id="rId22" display="https://ustaxcourt.gov/files/documents/rule-11.pdf" xr:uid="{5F18711A-BF79-430C-86E9-BB7BD02C3A77}"/>
-    <hyperlink ref="A13" r:id="rId23" display="https://www.ustaxcourt.gov/rules/limited_eoa/faq.pdf" xr:uid="{1B8D0982-7648-479A-AC85-E10144686AFA}"/>
-    <hyperlink ref="B13" r:id="rId24" display="https://ustaxcourt.gov/files/documents/lea_faq.pdf" xr:uid="{E0A3A479-9B71-4352-BCBF-6EC426E6EF9D}"/>
-    <hyperlink ref="A14" r:id="rId25" display="https://www.ustaxcourt.gov/todays-opinions" xr:uid="{63E278D2-99C9-497F-88D1-37787B44C468}"/>
-    <hyperlink ref="B14" r:id="rId26" xr:uid="{CA7B82AD-68E4-45D9-BCC6-895C7E6CEC33}"/>
-    <hyperlink ref="A15" r:id="rId27" display="https://www.ustaxcourt.gov/todays-orders" xr:uid="{1413C17D-7595-43B7-9A0D-1DF312C0C6EA}"/>
-    <hyperlink ref="B15" r:id="rId28" xr:uid="{8716BD67-EE4D-4EFB-A394-458921E334F4}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed spelling mistake in last update
</commit_message>
<xml_diff>
--- a/website/home/migrations/0115_create_redirects_for_broken_pdf_links.xlsx
+++ b/website/home/migrations/0115_create_redirects_for_broken_pdf_links.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30023"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F74BE9C8-A254-4ABD-B8FE-8B7164039CA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9BACBD6E-8D34-4323-9A0E-7A2C1F5D2268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
     <t>/clinics_academic_nonlaw_school.htm</t>
   </si>
   <si>
-    <t>/clinics-acadmic-non-law-school/</t>
+    <t>/clinics-academic-non-law-school/</t>
   </si>
   <si>
     <t>/clinics_nonacademic.htm</t>

</xml_diff>